<commit_message>
ALC corrections_still pending 2 points
</commit_message>
<xml_diff>
--- a/ALC/ALC - Asset Calculation Unit.xlsx
+++ b/ALC/ALC - Asset Calculation Unit.xlsx
@@ -43,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E9EEF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -87,13 +92,17 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of: 2026-07-09</t>
+          <t>As of: 2026-07-22</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -536,7 +545,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Term Months</t>
+          <t>Lifespan (months)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -576,116 +585,116 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>A1001</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>WWE</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Leasing</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Windblower</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="5" t="n">
         <v>46183</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="5" t="n">
         <v>46883</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="I4" t="n">
-        <v>23</v>
-      </c>
-      <c r="J4" s="5" t="n">
+      <c r="I4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J4" s="6" t="n">
         <v>9500</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="6" t="n">
         <v>10420</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="L4" s="6" t="n">
+        <v>475.97</v>
+      </c>
+      <c r="M4" s="6" t="n">
+        <v>9987.309999999999</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="O4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="M4" s="5" t="n">
-        <v>10420</v>
-      </c>
-      <c r="N4" s="6" t="n">
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>A1002</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>CHA</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Leasing</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Snow Blower</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>46194</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>47259</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>8200</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>8992</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>276.57</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>8752.780000000001</v>
+      </c>
+      <c r="N5" s="7" t="n">
         <v>0.051</v>
       </c>
-      <c r="O4" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>A1002</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>CHA</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Leasing</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Snow Blower</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>46194</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>47259</v>
-      </c>
-      <c r="H5" t="n">
-        <v>36</v>
-      </c>
-      <c r="I5" t="n">
-        <v>35</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>8200</v>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>8992</v>
-      </c>
-      <c r="L5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="5" t="n">
-        <v>8992</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>0.051</v>
-      </c>
-      <c r="O5" s="6" t="n">
+      <c r="O5" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -715,10 +724,10 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="8" t="n">
         <v>46198</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="8" t="n">
         <v>47628</v>
       </c>
       <c r="H6" t="n">
@@ -727,22 +736,22 @@
       <c r="I6" t="n">
         <v>47</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="9" t="n">
         <v>14000</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="9" t="n">
         <v>15340</v>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="L6" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="M6" s="5" t="n">
+      <c r="M6" s="9" t="n">
         <v>15340</v>
       </c>
-      <c r="N6" s="6" t="n">
+      <c r="N6" s="10" t="n">
         <v>0.051</v>
       </c>
-      <c r="O6" s="6" t="n">
+      <c r="O6" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -784,157 +793,157 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of: 2026-07-09 | Light gray rows = posted history</t>
+          <t>As of: 2026-07-22 | Light gray rows = posted history</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Asset ID</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>A1001</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Property ID</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>WWE</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Allocation</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Leasing</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Asset Description</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Windblower</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Lifecycle Status</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Asset Cost</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="13" t="n">
         <v>9500</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="13" t="n">
         <v>570</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Admin Expenses</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="13" t="n">
         <v>350</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Risk Cost Recovery</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="13" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Salvage Value</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="13" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Lease Base</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="13" t="n">
         <v>10420</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Salvage Periods</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Lifespan (months)</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="12" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>NIM (annual)</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -986,698 +995,698 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="8" t="n">
         <v>46183</v>
       </c>
       <c r="B20" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="10" t="n">
         <v>0.051</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="10" t="n">
         <v>0.004153777442692519</v>
       </c>
       <c r="E20" t="n">
         <v>23</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="9" t="n">
         <v>10420</v>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="G20" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="5" t="n">
+      <c r="H20" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="I20" s="9" t="n">
         <v>10420</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="5" t="n">
         <v>46213</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="7" t="n">
         <v>0.051</v>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="7" t="n">
         <v>0.00415378</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="6" t="n">
         <v>475.97</v>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="6" t="n">
         <v>43.28</v>
       </c>
-      <c r="H21" s="5" t="n">
+      <c r="H21" s="6" t="n">
         <v>432.69</v>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="I21" s="6" t="n">
         <v>9987.309999999999</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="B22" t="n">
         <v>2</v>
       </c>
-      <c r="C22" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D22" s="6" t="n">
+      <c r="C22" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D22" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E22" t="n">
         <v>22</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="G22" s="9" t="n">
         <v>43.07</v>
       </c>
-      <c r="H22" s="5" t="n">
+      <c r="H22" s="9" t="n">
         <v>433.75</v>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="I22" s="9" t="n">
         <v>9553.559999999999</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="8" t="n">
         <v>46275</v>
       </c>
       <c r="B23" t="n">
         <v>3</v>
       </c>
-      <c r="C23" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D23" s="6" t="n">
+      <c r="C23" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D23" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E23" t="n">
         <v>21</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G23" s="9" t="n">
         <v>41.2</v>
       </c>
-      <c r="H23" s="5" t="n">
+      <c r="H23" s="9" t="n">
         <v>435.62</v>
       </c>
-      <c r="I23" s="5" t="n">
+      <c r="I23" s="9" t="n">
         <v>9117.940000000001</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="8" t="n">
         <v>46305</v>
       </c>
       <c r="B24" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D24" s="6" t="n">
+      <c r="C24" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D24" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E24" t="n">
         <v>20</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="G24" s="9" t="n">
         <v>39.32</v>
       </c>
-      <c r="H24" s="5" t="n">
+      <c r="H24" s="9" t="n">
         <v>437.5</v>
       </c>
-      <c r="I24" s="5" t="n">
+      <c r="I24" s="9" t="n">
         <v>8680.440000000001</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="8" t="n">
         <v>46336</v>
       </c>
       <c r="B25" t="n">
         <v>5</v>
       </c>
-      <c r="C25" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D25" s="6" t="n">
+      <c r="C25" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D25" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E25" t="n">
         <v>19</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="G25" s="9" t="n">
         <v>37.44</v>
       </c>
-      <c r="H25" s="5" t="n">
+      <c r="H25" s="9" t="n">
         <v>439.39</v>
       </c>
-      <c r="I25" s="5" t="n">
-        <v>8241.059999999999</v>
+      <c r="I25" s="9" t="n">
+        <v>8241.049999999999</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="8" t="n">
         <v>46366</v>
       </c>
       <c r="B26" t="n">
         <v>6</v>
       </c>
-      <c r="C26" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D26" s="6" t="n">
+      <c r="C26" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D26" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E26" t="n">
         <v>18</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="G26" s="9" t="n">
         <v>35.54</v>
       </c>
-      <c r="H26" s="5" t="n">
+      <c r="H26" s="9" t="n">
         <v>441.28</v>
       </c>
-      <c r="I26" s="5" t="n">
-        <v>7799.78</v>
+      <c r="I26" s="9" t="n">
+        <v>7799.77</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="8" t="n">
         <v>46397</v>
       </c>
       <c r="B27" t="n">
         <v>7</v>
       </c>
-      <c r="C27" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D27" s="6" t="n">
+      <c r="C27" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D27" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E27" t="n">
         <v>17</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G27" s="9" t="n">
         <v>33.64</v>
       </c>
-      <c r="H27" s="5" t="n">
+      <c r="H27" s="9" t="n">
         <v>443.18</v>
       </c>
-      <c r="I27" s="5" t="n">
+      <c r="I27" s="9" t="n">
         <v>7356.59</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="8" t="n">
         <v>46428</v>
       </c>
       <c r="B28" t="n">
         <v>8</v>
       </c>
-      <c r="C28" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D28" s="6" t="n">
+      <c r="C28" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D28" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E28" t="n">
         <v>16</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G28" s="5" t="n">
+      <c r="G28" s="9" t="n">
         <v>31.73</v>
       </c>
-      <c r="H28" s="5" t="n">
+      <c r="H28" s="9" t="n">
         <v>445.1</v>
       </c>
-      <c r="I28" s="5" t="n">
-        <v>6911.5</v>
+      <c r="I28" s="9" t="n">
+        <v>6911.49</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="8" t="n">
         <v>46456</v>
       </c>
       <c r="B29" t="n">
         <v>9</v>
       </c>
-      <c r="C29" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D29" s="6" t="n">
+      <c r="C29" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D29" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E29" t="n">
         <v>15</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="G29" s="9" t="n">
         <v>29.81</v>
       </c>
-      <c r="H29" s="5" t="n">
+      <c r="H29" s="9" t="n">
         <v>447.02</v>
       </c>
-      <c r="I29" s="5" t="n">
+      <c r="I29" s="9" t="n">
         <v>6464.48</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="8" t="n">
         <v>46487</v>
       </c>
       <c r="B30" t="n">
         <v>10</v>
       </c>
-      <c r="C30" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D30" s="6" t="n">
+      <c r="C30" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D30" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E30" t="n">
         <v>14</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G30" s="5" t="n">
+      <c r="G30" s="9" t="n">
         <v>27.88</v>
       </c>
-      <c r="H30" s="5" t="n">
+      <c r="H30" s="9" t="n">
         <v>448.94</v>
       </c>
-      <c r="I30" s="5" t="n">
+      <c r="I30" s="9" t="n">
         <v>6015.54</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="8" t="n">
         <v>46517</v>
       </c>
       <c r="B31" t="n">
         <v>11</v>
       </c>
-      <c r="C31" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D31" s="6" t="n">
+      <c r="C31" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D31" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E31" t="n">
         <v>13</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G31" s="5" t="n">
+      <c r="G31" s="9" t="n">
         <v>25.94</v>
       </c>
-      <c r="H31" s="5" t="n">
+      <c r="H31" s="9" t="n">
         <v>450.88</v>
       </c>
-      <c r="I31" s="5" t="n">
+      <c r="I31" s="9" t="n">
         <v>5564.66</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="8" t="n">
         <v>46548</v>
       </c>
       <c r="B32" t="n">
         <v>12</v>
       </c>
-      <c r="C32" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D32" s="6" t="n">
+      <c r="C32" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D32" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E32" t="n">
         <v>12</v>
       </c>
-      <c r="F32" s="5" t="n">
+      <c r="F32" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G32" s="5" t="n">
+      <c r="G32" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="H32" s="5" t="n">
+      <c r="H32" s="9" t="n">
         <v>452.82</v>
       </c>
-      <c r="I32" s="5" t="n">
+      <c r="I32" s="9" t="n">
         <v>5111.83</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="8" t="n">
         <v>46578</v>
       </c>
       <c r="B33" t="n">
         <v>13</v>
       </c>
-      <c r="C33" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D33" s="6" t="n">
+      <c r="C33" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D33" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E33" t="n">
         <v>11</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F33" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="G33" s="9" t="n">
         <v>22.05</v>
       </c>
-      <c r="H33" s="5" t="n">
+      <c r="H33" s="9" t="n">
         <v>454.78</v>
       </c>
-      <c r="I33" s="5" t="n">
-        <v>4657.06</v>
+      <c r="I33" s="9" t="n">
+        <v>4657.05</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="A34" s="8" t="n">
         <v>46609</v>
       </c>
       <c r="B34" t="n">
         <v>14</v>
       </c>
-      <c r="C34" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D34" s="6" t="n">
+      <c r="C34" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D34" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E34" t="n">
         <v>10</v>
       </c>
-      <c r="F34" s="5" t="n">
+      <c r="F34" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G34" s="5" t="n">
+      <c r="G34" s="9" t="n">
         <v>20.09</v>
       </c>
-      <c r="H34" s="5" t="n">
+      <c r="H34" s="9" t="n">
         <v>456.74</v>
       </c>
-      <c r="I34" s="5" t="n">
+      <c r="I34" s="9" t="n">
         <v>4200.32</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n">
+      <c r="A35" s="8" t="n">
         <v>46640</v>
       </c>
       <c r="B35" t="n">
         <v>15</v>
       </c>
-      <c r="C35" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D35" s="6" t="n">
+      <c r="C35" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D35" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E35" t="n">
         <v>9</v>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="9" t="n">
         <v>18.12</v>
       </c>
-      <c r="H35" s="5" t="n">
+      <c r="H35" s="9" t="n">
         <v>458.71</v>
       </c>
-      <c r="I35" s="5" t="n">
+      <c r="I35" s="9" t="n">
         <v>3741.61</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="8" t="n">
         <v>46670</v>
       </c>
       <c r="B36" t="n">
         <v>16</v>
       </c>
-      <c r="C36" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D36" s="6" t="n">
+      <c r="C36" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D36" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E36" t="n">
         <v>8</v>
       </c>
-      <c r="F36" s="5" t="n">
+      <c r="F36" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G36" s="5" t="n">
+      <c r="G36" s="9" t="n">
         <v>16.14</v>
       </c>
-      <c r="H36" s="5" t="n">
+      <c r="H36" s="9" t="n">
         <v>460.69</v>
       </c>
-      <c r="I36" s="5" t="n">
+      <c r="I36" s="9" t="n">
         <v>3280.92</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n">
+      <c r="A37" s="8" t="n">
         <v>46701</v>
       </c>
       <c r="B37" t="n">
         <v>17</v>
       </c>
-      <c r="C37" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D37" s="6" t="n">
+      <c r="C37" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D37" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E37" t="n">
         <v>7</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F37" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="G37" s="9" t="n">
         <v>14.15</v>
       </c>
-      <c r="H37" s="5" t="n">
+      <c r="H37" s="9" t="n">
         <v>462.67</v>
       </c>
-      <c r="I37" s="5" t="n">
+      <c r="I37" s="9" t="n">
         <v>2818.25</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n">
+      <c r="A38" s="8" t="n">
         <v>46731</v>
       </c>
       <c r="B38" t="n">
         <v>18</v>
       </c>
-      <c r="C38" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D38" s="6" t="n">
+      <c r="C38" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D38" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E38" t="n">
         <v>6</v>
       </c>
-      <c r="F38" s="5" t="n">
+      <c r="F38" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G38" s="5" t="n">
+      <c r="G38" s="9" t="n">
         <v>12.15</v>
       </c>
-      <c r="H38" s="5" t="n">
+      <c r="H38" s="9" t="n">
         <v>464.67</v>
       </c>
-      <c r="I38" s="5" t="n">
+      <c r="I38" s="9" t="n">
         <v>2353.58</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n">
+      <c r="A39" s="8" t="n">
         <v>46762</v>
       </c>
       <c r="B39" t="n">
         <v>19</v>
       </c>
-      <c r="C39" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D39" s="6" t="n">
+      <c r="C39" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D39" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E39" t="n">
         <v>5</v>
       </c>
-      <c r="F39" s="5" t="n">
+      <c r="F39" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G39" s="5" t="n">
+      <c r="G39" s="9" t="n">
         <v>10.15</v>
       </c>
-      <c r="H39" s="5" t="n">
+      <c r="H39" s="9" t="n">
         <v>466.67</v>
       </c>
-      <c r="I39" s="5" t="n">
+      <c r="I39" s="9" t="n">
         <v>1886.91</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n">
+      <c r="A40" s="8" t="n">
         <v>46793</v>
       </c>
       <c r="B40" t="n">
         <v>20</v>
       </c>
-      <c r="C40" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D40" s="6" t="n">
+      <c r="C40" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D40" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E40" t="n">
         <v>4</v>
       </c>
-      <c r="F40" s="5" t="n">
+      <c r="F40" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G40" s="5" t="n">
+      <c r="G40" s="9" t="n">
         <v>8.140000000000001</v>
       </c>
-      <c r="H40" s="5" t="n">
+      <c r="H40" s="9" t="n">
         <v>468.69</v>
       </c>
-      <c r="I40" s="5" t="n">
+      <c r="I40" s="9" t="n">
         <v>1418.22</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n">
+      <c r="A41" s="8" t="n">
         <v>46822</v>
       </c>
       <c r="B41" t="n">
         <v>21</v>
       </c>
-      <c r="C41" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D41" s="6" t="n">
+      <c r="C41" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D41" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E41" t="n">
         <v>3</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F41" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G41" s="5" t="n">
+      <c r="G41" s="9" t="n">
         <v>6.12</v>
       </c>
-      <c r="H41" s="5" t="n">
+      <c r="H41" s="9" t="n">
         <v>470.71</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I41" s="9" t="n">
         <v>947.51</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n">
+      <c r="A42" s="8" t="n">
         <v>46853</v>
       </c>
       <c r="B42" t="n">
         <v>22</v>
       </c>
-      <c r="C42" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D42" s="6" t="n">
+      <c r="C42" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D42" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>
       </c>
-      <c r="F42" s="5" t="n">
+      <c r="F42" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G42" s="5" t="n">
+      <c r="G42" s="9" t="n">
         <v>4.09</v>
       </c>
-      <c r="H42" s="5" t="n">
+      <c r="H42" s="9" t="n">
         <v>472.74</v>
       </c>
-      <c r="I42" s="5" t="n">
+      <c r="I42" s="9" t="n">
         <v>474.78</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n">
+      <c r="A43" s="8" t="n">
         <v>46883</v>
       </c>
       <c r="B43" t="n">
         <v>23</v>
       </c>
-      <c r="C43" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D43" s="6" t="n">
+      <c r="C43" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D43" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E43" t="n">
         <v>1</v>
       </c>
-      <c r="F43" s="5" t="n">
+      <c r="F43" s="9" t="n">
         <v>476.82</v>
       </c>
-      <c r="G43" s="5" t="n">
+      <c r="G43" s="9" t="n">
         <v>2.05</v>
       </c>
-      <c r="H43" s="5" t="n">
+      <c r="H43" s="9" t="n">
         <v>474.78</v>
       </c>
-      <c r="I43" s="5" t="n">
+      <c r="I43" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1719,157 +1728,157 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of: 2026-07-09 | Light gray rows = posted history</t>
+          <t>As of: 2026-07-22 | Light gray rows = posted history</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Asset ID</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>A1002</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Property ID</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Allocation</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Leasing</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Asset Description</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Snow Blower</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Lifecycle Status</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Asset Cost</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="13" t="n">
         <v>8200</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="13" t="n">
         <v>492</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Admin Expenses</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="13" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Risk Cost Recovery</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="13" t="n">
         <v>260</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Salvage Value</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="13" t="n">
         <v>260</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Lease Base</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="13" t="n">
         <v>8992</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Salvage Periods</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Lifespan (months)</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="12" t="n">
         <v>36</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>NIM (annual)</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1921,1046 +1930,1046 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="8" t="n">
         <v>46194</v>
       </c>
       <c r="B20" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="10" t="n">
         <v>0.051</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="10" t="n">
         <v>0.004153777442692519</v>
       </c>
       <c r="E20" t="n">
         <v>35</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="9" t="n">
         <v>8992</v>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="G20" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="5" t="n">
+      <c r="H20" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="I20" s="9" t="n">
         <v>8992</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="5" t="n">
         <v>46224</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="7" t="n">
         <v>0.051</v>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="7" t="n">
         <v>0.00415378</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="6" t="n">
         <v>276.57</v>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="6" t="n">
         <v>37.35</v>
       </c>
-      <c r="H21" s="5" t="n">
+      <c r="H21" s="6" t="n">
         <v>239.22</v>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="I21" s="6" t="n">
         <v>8752.780000000001</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="8" t="n">
         <v>46255</v>
       </c>
       <c r="B22" t="n">
         <v>2</v>
       </c>
-      <c r="C22" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D22" s="6" t="n">
+      <c r="C22" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D22" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E22" t="n">
         <v>34</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="G22" s="9" t="n">
         <v>37.75</v>
       </c>
-      <c r="H22" s="5" t="n">
+      <c r="H22" s="9" t="n">
         <v>239.57</v>
       </c>
-      <c r="I22" s="5" t="n">
-        <v>8513.200000000001</v>
+      <c r="I22" s="9" t="n">
+        <v>8513.209999999999</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="8" t="n">
         <v>46286</v>
       </c>
       <c r="B23" t="n">
         <v>3</v>
       </c>
-      <c r="C23" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D23" s="6" t="n">
+      <c r="C23" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D23" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E23" t="n">
         <v>33</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G23" s="9" t="n">
         <v>36.72</v>
       </c>
-      <c r="H23" s="5" t="n">
+      <c r="H23" s="9" t="n">
         <v>240.61</v>
       </c>
-      <c r="I23" s="5" t="n">
-        <v>8272.59</v>
+      <c r="I23" s="9" t="n">
+        <v>8272.6</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="8" t="n">
         <v>46316</v>
       </c>
       <c r="B24" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D24" s="6" t="n">
+      <c r="C24" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D24" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E24" t="n">
         <v>32</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="G24" s="9" t="n">
         <v>35.68</v>
       </c>
-      <c r="H24" s="5" t="n">
+      <c r="H24" s="9" t="n">
         <v>241.65</v>
       </c>
-      <c r="I24" s="5" t="n">
+      <c r="I24" s="9" t="n">
         <v>8030.95</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="8" t="n">
         <v>46347</v>
       </c>
       <c r="B25" t="n">
         <v>5</v>
       </c>
-      <c r="C25" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D25" s="6" t="n">
+      <c r="C25" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D25" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E25" t="n">
         <v>31</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="G25" s="9" t="n">
         <v>34.64</v>
       </c>
-      <c r="H25" s="5" t="n">
+      <c r="H25" s="9" t="n">
         <v>242.69</v>
       </c>
-      <c r="I25" s="5" t="n">
+      <c r="I25" s="9" t="n">
         <v>7788.26</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="8" t="n">
         <v>46377</v>
       </c>
       <c r="B26" t="n">
         <v>6</v>
       </c>
-      <c r="C26" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D26" s="6" t="n">
+      <c r="C26" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D26" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E26" t="n">
         <v>30</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="G26" s="9" t="n">
         <v>33.59</v>
       </c>
-      <c r="H26" s="5" t="n">
+      <c r="H26" s="9" t="n">
         <v>243.73</v>
       </c>
-      <c r="I26" s="5" t="n">
+      <c r="I26" s="9" t="n">
         <v>7544.53</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="8" t="n">
         <v>46408</v>
       </c>
       <c r="B27" t="n">
         <v>7</v>
       </c>
-      <c r="C27" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D27" s="6" t="n">
+      <c r="C27" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D27" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E27" t="n">
         <v>29</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G27" s="9" t="n">
         <v>32.54</v>
       </c>
-      <c r="H27" s="5" t="n">
+      <c r="H27" s="9" t="n">
         <v>244.79</v>
       </c>
-      <c r="I27" s="5" t="n">
+      <c r="I27" s="9" t="n">
         <v>7299.74</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="8" t="n">
         <v>46439</v>
       </c>
       <c r="B28" t="n">
         <v>8</v>
       </c>
-      <c r="C28" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D28" s="6" t="n">
+      <c r="C28" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D28" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E28" t="n">
         <v>28</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G28" s="5" t="n">
+      <c r="G28" s="9" t="n">
         <v>31.48</v>
       </c>
-      <c r="H28" s="5" t="n">
+      <c r="H28" s="9" t="n">
         <v>245.84</v>
       </c>
-      <c r="I28" s="5" t="n">
+      <c r="I28" s="9" t="n">
         <v>7053.9</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="8" t="n">
         <v>46467</v>
       </c>
       <c r="B29" t="n">
         <v>9</v>
       </c>
-      <c r="C29" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D29" s="6" t="n">
+      <c r="C29" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D29" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E29" t="n">
         <v>27</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="G29" s="9" t="n">
         <v>30.42</v>
       </c>
-      <c r="H29" s="5" t="n">
+      <c r="H29" s="9" t="n">
         <v>246.9</v>
       </c>
-      <c r="I29" s="5" t="n">
+      <c r="I29" s="9" t="n">
         <v>6807</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="8" t="n">
         <v>46498</v>
       </c>
       <c r="B30" t="n">
         <v>10</v>
       </c>
-      <c r="C30" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D30" s="6" t="n">
+      <c r="C30" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D30" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E30" t="n">
         <v>26</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G30" s="5" t="n">
+      <c r="G30" s="9" t="n">
         <v>29.36</v>
       </c>
-      <c r="H30" s="5" t="n">
+      <c r="H30" s="9" t="n">
         <v>247.97</v>
       </c>
-      <c r="I30" s="5" t="n">
+      <c r="I30" s="9" t="n">
         <v>6559.03</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="8" t="n">
         <v>46528</v>
       </c>
       <c r="B31" t="n">
         <v>11</v>
       </c>
-      <c r="C31" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D31" s="6" t="n">
+      <c r="C31" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D31" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E31" t="n">
         <v>25</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G31" s="5" t="n">
+      <c r="G31" s="9" t="n">
         <v>28.29</v>
       </c>
-      <c r="H31" s="5" t="n">
+      <c r="H31" s="9" t="n">
         <v>249.04</v>
       </c>
-      <c r="I31" s="5" t="n">
-        <v>6309.99</v>
+      <c r="I31" s="9" t="n">
+        <v>6310</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="8" t="n">
         <v>46559</v>
       </c>
       <c r="B32" t="n">
         <v>12</v>
       </c>
-      <c r="C32" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D32" s="6" t="n">
+      <c r="C32" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D32" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E32" t="n">
         <v>24</v>
       </c>
-      <c r="F32" s="5" t="n">
+      <c r="F32" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G32" s="5" t="n">
+      <c r="G32" s="9" t="n">
         <v>27.21</v>
       </c>
-      <c r="H32" s="5" t="n">
+      <c r="H32" s="9" t="n">
         <v>250.11</v>
       </c>
-      <c r="I32" s="5" t="n">
-        <v>6059.88</v>
+      <c r="I32" s="9" t="n">
+        <v>6059.89</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="8" t="n">
         <v>46589</v>
       </c>
       <c r="B33" t="n">
         <v>13</v>
       </c>
-      <c r="C33" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D33" s="6" t="n">
+      <c r="C33" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D33" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E33" t="n">
         <v>23</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F33" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="G33" s="9" t="n">
         <v>26.14</v>
       </c>
-      <c r="H33" s="5" t="n">
+      <c r="H33" s="9" t="n">
         <v>251.19</v>
       </c>
-      <c r="I33" s="5" t="n">
+      <c r="I33" s="9" t="n">
         <v>5808.7</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="A34" s="8" t="n">
         <v>46620</v>
       </c>
       <c r="B34" t="n">
         <v>14</v>
       </c>
-      <c r="C34" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D34" s="6" t="n">
+      <c r="C34" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D34" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E34" t="n">
         <v>22</v>
       </c>
-      <c r="F34" s="5" t="n">
+      <c r="F34" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G34" s="5" t="n">
+      <c r="G34" s="9" t="n">
         <v>25.05</v>
       </c>
-      <c r="H34" s="5" t="n">
+      <c r="H34" s="9" t="n">
         <v>252.27</v>
       </c>
-      <c r="I34" s="5" t="n">
-        <v>5556.42</v>
+      <c r="I34" s="9" t="n">
+        <v>5556.43</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n">
+      <c r="A35" s="8" t="n">
         <v>46651</v>
       </c>
       <c r="B35" t="n">
         <v>15</v>
       </c>
-      <c r="C35" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D35" s="6" t="n">
+      <c r="C35" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D35" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E35" t="n">
         <v>21</v>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="9" t="n">
         <v>23.96</v>
       </c>
-      <c r="H35" s="5" t="n">
+      <c r="H35" s="9" t="n">
         <v>253.36</v>
       </c>
-      <c r="I35" s="5" t="n">
-        <v>5303.06</v>
+      <c r="I35" s="9" t="n">
+        <v>5303.07</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="8" t="n">
         <v>46681</v>
       </c>
       <c r="B36" t="n">
         <v>16</v>
       </c>
-      <c r="C36" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D36" s="6" t="n">
+      <c r="C36" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D36" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E36" t="n">
         <v>20</v>
       </c>
-      <c r="F36" s="5" t="n">
+      <c r="F36" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G36" s="5" t="n">
+      <c r="G36" s="9" t="n">
         <v>22.87</v>
       </c>
-      <c r="H36" s="5" t="n">
+      <c r="H36" s="9" t="n">
         <v>254.45</v>
       </c>
-      <c r="I36" s="5" t="n">
+      <c r="I36" s="9" t="n">
         <v>5048.61</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n">
+      <c r="A37" s="8" t="n">
         <v>46712</v>
       </c>
       <c r="B37" t="n">
         <v>17</v>
       </c>
-      <c r="C37" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D37" s="6" t="n">
+      <c r="C37" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D37" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E37" t="n">
         <v>19</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F37" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="G37" s="9" t="n">
         <v>21.77</v>
       </c>
-      <c r="H37" s="5" t="n">
+      <c r="H37" s="9" t="n">
         <v>255.55</v>
       </c>
-      <c r="I37" s="5" t="n">
+      <c r="I37" s="9" t="n">
         <v>4793.06</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n">
+      <c r="A38" s="8" t="n">
         <v>46742</v>
       </c>
       <c r="B38" t="n">
         <v>18</v>
       </c>
-      <c r="C38" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D38" s="6" t="n">
+      <c r="C38" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D38" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E38" t="n">
         <v>18</v>
       </c>
-      <c r="F38" s="5" t="n">
+      <c r="F38" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G38" s="5" t="n">
+      <c r="G38" s="9" t="n">
         <v>20.67</v>
       </c>
-      <c r="H38" s="5" t="n">
+      <c r="H38" s="9" t="n">
         <v>256.65</v>
       </c>
-      <c r="I38" s="5" t="n">
+      <c r="I38" s="9" t="n">
         <v>4536.41</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n">
+      <c r="A39" s="8" t="n">
         <v>46773</v>
       </c>
       <c r="B39" t="n">
         <v>19</v>
       </c>
-      <c r="C39" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D39" s="6" t="n">
+      <c r="C39" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D39" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E39" t="n">
         <v>17</v>
       </c>
-      <c r="F39" s="5" t="n">
+      <c r="F39" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G39" s="5" t="n">
+      <c r="G39" s="9" t="n">
         <v>19.56</v>
       </c>
-      <c r="H39" s="5" t="n">
+      <c r="H39" s="9" t="n">
         <v>257.76</v>
       </c>
-      <c r="I39" s="5" t="n">
+      <c r="I39" s="9" t="n">
         <v>4278.65</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n">
+      <c r="A40" s="8" t="n">
         <v>46804</v>
       </c>
       <c r="B40" t="n">
         <v>20</v>
       </c>
-      <c r="C40" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D40" s="6" t="n">
+      <c r="C40" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D40" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E40" t="n">
         <v>16</v>
       </c>
-      <c r="F40" s="5" t="n">
+      <c r="F40" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G40" s="5" t="n">
+      <c r="G40" s="9" t="n">
         <v>18.45</v>
       </c>
-      <c r="H40" s="5" t="n">
+      <c r="H40" s="9" t="n">
         <v>258.87</v>
       </c>
-      <c r="I40" s="5" t="n">
+      <c r="I40" s="9" t="n">
         <v>4019.78</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n">
+      <c r="A41" s="8" t="n">
         <v>46833</v>
       </c>
       <c r="B41" t="n">
         <v>21</v>
       </c>
-      <c r="C41" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D41" s="6" t="n">
+      <c r="C41" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D41" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E41" t="n">
         <v>15</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F41" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G41" s="5" t="n">
+      <c r="G41" s="9" t="n">
         <v>17.34</v>
       </c>
-      <c r="H41" s="5" t="n">
+      <c r="H41" s="9" t="n">
         <v>259.99</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I41" s="9" t="n">
         <v>3759.79</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n">
+      <c r="A42" s="8" t="n">
         <v>46864</v>
       </c>
       <c r="B42" t="n">
         <v>22</v>
       </c>
-      <c r="C42" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D42" s="6" t="n">
+      <c r="C42" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D42" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E42" t="n">
         <v>14</v>
       </c>
-      <c r="F42" s="5" t="n">
+      <c r="F42" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G42" s="5" t="n">
+      <c r="G42" s="9" t="n">
         <v>16.22</v>
       </c>
-      <c r="H42" s="5" t="n">
+      <c r="H42" s="9" t="n">
         <v>261.11</v>
       </c>
-      <c r="I42" s="5" t="n">
+      <c r="I42" s="9" t="n">
         <v>3498.68</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n">
+      <c r="A43" s="8" t="n">
         <v>46894</v>
       </c>
       <c r="B43" t="n">
         <v>23</v>
       </c>
-      <c r="C43" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D43" s="6" t="n">
+      <c r="C43" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D43" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E43" t="n">
         <v>13</v>
       </c>
-      <c r="F43" s="5" t="n">
+      <c r="F43" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G43" s="5" t="n">
+      <c r="G43" s="9" t="n">
         <v>15.09</v>
       </c>
-      <c r="H43" s="5" t="n">
-        <v>262.23</v>
-      </c>
-      <c r="I43" s="5" t="n">
+      <c r="H43" s="9" t="n">
+        <v>262.24</v>
+      </c>
+      <c r="I43" s="9" t="n">
         <v>3236.45</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="n">
+      <c r="A44" s="8" t="n">
         <v>46925</v>
       </c>
       <c r="B44" t="n">
         <v>24</v>
       </c>
-      <c r="C44" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D44" s="6" t="n">
+      <c r="C44" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D44" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E44" t="n">
         <v>12</v>
       </c>
-      <c r="F44" s="5" t="n">
+      <c r="F44" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G44" s="5" t="n">
+      <c r="G44" s="9" t="n">
         <v>13.96</v>
       </c>
-      <c r="H44" s="5" t="n">
+      <c r="H44" s="9" t="n">
         <v>263.37</v>
       </c>
-      <c r="I44" s="5" t="n">
+      <c r="I44" s="9" t="n">
         <v>2973.08</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n">
+      <c r="A45" s="8" t="n">
         <v>46955</v>
       </c>
       <c r="B45" t="n">
         <v>25</v>
       </c>
-      <c r="C45" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D45" s="6" t="n">
+      <c r="C45" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D45" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E45" t="n">
         <v>11</v>
       </c>
-      <c r="F45" s="5" t="n">
+      <c r="F45" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G45" s="5" t="n">
+      <c r="G45" s="9" t="n">
         <v>12.82</v>
       </c>
-      <c r="H45" s="5" t="n">
+      <c r="H45" s="9" t="n">
         <v>264.5</v>
       </c>
-      <c r="I45" s="5" t="n">
+      <c r="I45" s="9" t="n">
         <v>2708.58</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="A46" s="8" t="n">
         <v>46986</v>
       </c>
       <c r="B46" t="n">
         <v>26</v>
       </c>
-      <c r="C46" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D46" s="6" t="n">
+      <c r="C46" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D46" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E46" t="n">
         <v>10</v>
       </c>
-      <c r="F46" s="5" t="n">
+      <c r="F46" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G46" s="5" t="n">
+      <c r="G46" s="9" t="n">
         <v>11.68</v>
       </c>
-      <c r="H46" s="5" t="n">
+      <c r="H46" s="9" t="n">
         <v>265.64</v>
       </c>
-      <c r="I46" s="5" t="n">
+      <c r="I46" s="9" t="n">
         <v>2442.94</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="n">
+      <c r="A47" s="8" t="n">
         <v>47017</v>
       </c>
       <c r="B47" t="n">
         <v>27</v>
       </c>
-      <c r="C47" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D47" s="6" t="n">
+      <c r="C47" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D47" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E47" t="n">
         <v>9</v>
       </c>
-      <c r="F47" s="5" t="n">
+      <c r="F47" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G47" s="5" t="n">
+      <c r="G47" s="9" t="n">
         <v>10.54</v>
       </c>
-      <c r="H47" s="5" t="n">
+      <c r="H47" s="9" t="n">
         <v>266.79</v>
       </c>
-      <c r="I47" s="5" t="n">
+      <c r="I47" s="9" t="n">
         <v>2176.15</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n">
+      <c r="A48" s="8" t="n">
         <v>47047</v>
       </c>
       <c r="B48" t="n">
         <v>28</v>
       </c>
-      <c r="C48" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D48" s="6" t="n">
+      <c r="C48" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D48" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E48" t="n">
         <v>8</v>
       </c>
-      <c r="F48" s="5" t="n">
+      <c r="F48" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G48" s="5" t="n">
+      <c r="G48" s="9" t="n">
         <v>9.390000000000001</v>
       </c>
-      <c r="H48" s="5" t="n">
+      <c r="H48" s="9" t="n">
         <v>267.94</v>
       </c>
-      <c r="I48" s="5" t="n">
+      <c r="I48" s="9" t="n">
         <v>1908.21</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="n">
+      <c r="A49" s="8" t="n">
         <v>47078</v>
       </c>
       <c r="B49" t="n">
         <v>29</v>
       </c>
-      <c r="C49" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D49" s="6" t="n">
+      <c r="C49" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D49" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E49" t="n">
         <v>7</v>
       </c>
-      <c r="F49" s="5" t="n">
+      <c r="F49" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G49" s="5" t="n">
+      <c r="G49" s="9" t="n">
         <v>8.23</v>
       </c>
-      <c r="H49" s="5" t="n">
+      <c r="H49" s="9" t="n">
         <v>269.09</v>
       </c>
-      <c r="I49" s="5" t="n">
-        <v>1639.11</v>
+      <c r="I49" s="9" t="n">
+        <v>1639.12</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n">
+      <c r="A50" s="8" t="n">
         <v>47108</v>
       </c>
       <c r="B50" t="n">
         <v>30</v>
       </c>
-      <c r="C50" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D50" s="6" t="n">
+      <c r="C50" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D50" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E50" t="n">
         <v>6</v>
       </c>
-      <c r="F50" s="5" t="n">
+      <c r="F50" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G50" s="5" t="n">
+      <c r="G50" s="9" t="n">
         <v>7.07</v>
       </c>
-      <c r="H50" s="5" t="n">
+      <c r="H50" s="9" t="n">
         <v>270.26</v>
       </c>
-      <c r="I50" s="5" t="n">
+      <c r="I50" s="9" t="n">
         <v>1368.86</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n">
+      <c r="A51" s="8" t="n">
         <v>47139</v>
       </c>
       <c r="B51" t="n">
         <v>31</v>
       </c>
-      <c r="C51" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D51" s="6" t="n">
+      <c r="C51" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D51" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E51" t="n">
         <v>5</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F51" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G51" s="5" t="n">
+      <c r="G51" s="9" t="n">
         <v>5.9</v>
       </c>
-      <c r="H51" s="5" t="n">
+      <c r="H51" s="9" t="n">
         <v>271.42</v>
       </c>
-      <c r="I51" s="5" t="n">
+      <c r="I51" s="9" t="n">
         <v>1097.44</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="n">
+      <c r="A52" s="8" t="n">
         <v>47170</v>
       </c>
       <c r="B52" t="n">
         <v>32</v>
       </c>
-      <c r="C52" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D52" s="6" t="n">
+      <c r="C52" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D52" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E52" t="n">
         <v>4</v>
       </c>
-      <c r="F52" s="5" t="n">
+      <c r="F52" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G52" s="5" t="n">
+      <c r="G52" s="9" t="n">
         <v>4.73</v>
       </c>
-      <c r="H52" s="5" t="n">
+      <c r="H52" s="9" t="n">
         <v>272.59</v>
       </c>
-      <c r="I52" s="5" t="n">
+      <c r="I52" s="9" t="n">
         <v>824.85</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="n">
+      <c r="A53" s="8" t="n">
         <v>47198</v>
       </c>
       <c r="B53" t="n">
         <v>33</v>
       </c>
-      <c r="C53" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D53" s="6" t="n">
+      <c r="C53" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D53" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E53" t="n">
         <v>3</v>
       </c>
-      <c r="F53" s="5" t="n">
+      <c r="F53" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G53" s="5" t="n">
+      <c r="G53" s="9" t="n">
         <v>3.56</v>
       </c>
-      <c r="H53" s="5" t="n">
+      <c r="H53" s="9" t="n">
         <v>273.77</v>
       </c>
-      <c r="I53" s="5" t="n">
+      <c r="I53" s="9" t="n">
         <v>551.08</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="n">
+      <c r="A54" s="8" t="n">
         <v>47229</v>
       </c>
       <c r="B54" t="n">
         <v>34</v>
       </c>
-      <c r="C54" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D54" s="6" t="n">
+      <c r="C54" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D54" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E54" t="n">
         <v>2</v>
       </c>
-      <c r="F54" s="5" t="n">
+      <c r="F54" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G54" s="5" t="n">
+      <c r="G54" s="9" t="n">
         <v>2.38</v>
       </c>
-      <c r="H54" s="5" t="n">
+      <c r="H54" s="9" t="n">
         <v>274.95</v>
       </c>
-      <c r="I54" s="5" t="n">
+      <c r="I54" s="9" t="n">
         <v>276.13</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="n">
+      <c r="A55" s="8" t="n">
         <v>47259</v>
       </c>
       <c r="B55" t="n">
         <v>35</v>
       </c>
-      <c r="C55" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D55" s="6" t="n">
+      <c r="C55" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D55" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E55" t="n">
         <v>1</v>
       </c>
-      <c r="F55" s="5" t="n">
+      <c r="F55" s="9" t="n">
         <v>277.32</v>
       </c>
-      <c r="G55" s="5" t="n">
+      <c r="G55" s="9" t="n">
         <v>1.19</v>
       </c>
-      <c r="H55" s="5" t="n">
+      <c r="H55" s="9" t="n">
         <v>276.13</v>
       </c>
-      <c r="I55" s="5" t="n">
+      <c r="I55" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3002,157 +3011,157 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of: 2026-07-09 | Light gray rows = posted history</t>
+          <t>As of: 2026-07-22 | Light gray rows = posted history</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Asset ID</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>A1003</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Property ID</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>LPA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Allocation</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Leasing</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Asset Description</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Golf Cart</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Lifecycle Status</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Asset Cost</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="13" t="n">
         <v>14000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="13" t="n">
         <v>840</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Admin Expenses</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="13" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Risk Cost Recovery</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="13" t="n">
         <v>420</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Salvage Value</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="13" t="n">
         <v>420</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Lease Base</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="13" t="n">
         <v>15340</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Salvage Periods</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Lifespan (months)</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="12" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>NIM (annual)</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3204,1394 +3213,1394 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="8" t="n">
         <v>46198</v>
       </c>
       <c r="B20" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="10" t="n">
         <v>0.051</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="10" t="n">
         <v>0.004153777442692519</v>
       </c>
       <c r="E20" t="n">
         <v>47</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="9" t="n">
         <v>15340</v>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="G20" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="5" t="n">
+      <c r="H20" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="I20" s="9" t="n">
         <v>15340</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="8" t="n">
         <v>46228</v>
       </c>
       <c r="B21" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="10" t="n">
         <v>0.051</v>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="10" t="n">
         <v>0.00415378</v>
       </c>
       <c r="E21" t="n">
         <v>47</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="9" t="n">
         <v>359.95</v>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="9" t="n">
         <v>63.72</v>
       </c>
-      <c r="H21" s="5" t="n">
+      <c r="H21" s="9" t="n">
         <v>296.23</v>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="I21" s="9" t="n">
         <v>15043.77</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="8" t="n">
         <v>46259</v>
       </c>
       <c r="B22" t="n">
         <v>2</v>
       </c>
-      <c r="C22" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D22" s="6" t="n">
+      <c r="C22" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D22" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E22" t="n">
         <v>46</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="G22" s="9" t="n">
         <v>64.88</v>
       </c>
-      <c r="H22" s="5" t="n">
+      <c r="H22" s="9" t="n">
         <v>296.37</v>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="I22" s="9" t="n">
         <v>14747.39</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="8" t="n">
         <v>46290</v>
       </c>
       <c r="B23" t="n">
         <v>3</v>
       </c>
-      <c r="C23" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D23" s="6" t="n">
+      <c r="C23" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D23" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E23" t="n">
         <v>45</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G23" s="9" t="n">
         <v>63.6</v>
       </c>
-      <c r="H23" s="5" t="n">
+      <c r="H23" s="9" t="n">
         <v>297.65</v>
       </c>
-      <c r="I23" s="5" t="n">
+      <c r="I23" s="9" t="n">
         <v>14449.74</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="8" t="n">
         <v>46320</v>
       </c>
       <c r="B24" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D24" s="6" t="n">
+      <c r="C24" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D24" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E24" t="n">
         <v>44</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="G24" s="9" t="n">
         <v>62.32</v>
       </c>
-      <c r="H24" s="5" t="n">
+      <c r="H24" s="9" t="n">
         <v>298.93</v>
       </c>
-      <c r="I24" s="5" t="n">
+      <c r="I24" s="9" t="n">
         <v>14150.81</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="8" t="n">
         <v>46351</v>
       </c>
       <c r="B25" t="n">
         <v>5</v>
       </c>
-      <c r="C25" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D25" s="6" t="n">
+      <c r="C25" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D25" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E25" t="n">
         <v>43</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="G25" s="9" t="n">
         <v>61.03</v>
       </c>
-      <c r="H25" s="5" t="n">
+      <c r="H25" s="9" t="n">
         <v>300.22</v>
       </c>
-      <c r="I25" s="5" t="n">
+      <c r="I25" s="9" t="n">
         <v>13850.59</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="8" t="n">
         <v>46381</v>
       </c>
       <c r="B26" t="n">
         <v>6</v>
       </c>
-      <c r="C26" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D26" s="6" t="n">
+      <c r="C26" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D26" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E26" t="n">
         <v>42</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="G26" s="9" t="n">
         <v>59.74</v>
       </c>
-      <c r="H26" s="5" t="n">
+      <c r="H26" s="9" t="n">
         <v>301.52</v>
       </c>
-      <c r="I26" s="5" t="n">
+      <c r="I26" s="9" t="n">
         <v>13549.07</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="8" t="n">
         <v>46412</v>
       </c>
       <c r="B27" t="n">
         <v>7</v>
       </c>
-      <c r="C27" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D27" s="6" t="n">
+      <c r="C27" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D27" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E27" t="n">
         <v>41</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G27" s="9" t="n">
         <v>58.44</v>
       </c>
-      <c r="H27" s="5" t="n">
+      <c r="H27" s="9" t="n">
         <v>302.82</v>
       </c>
-      <c r="I27" s="5" t="n">
+      <c r="I27" s="9" t="n">
         <v>13246.25</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="8" t="n">
         <v>46443</v>
       </c>
       <c r="B28" t="n">
         <v>8</v>
       </c>
-      <c r="C28" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D28" s="6" t="n">
+      <c r="C28" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D28" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E28" t="n">
         <v>40</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G28" s="5" t="n">
+      <c r="G28" s="9" t="n">
         <v>57.13</v>
       </c>
-      <c r="H28" s="5" t="n">
+      <c r="H28" s="9" t="n">
         <v>304.12</v>
       </c>
-      <c r="I28" s="5" t="n">
+      <c r="I28" s="9" t="n">
         <v>12942.13</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="8" t="n">
         <v>46471</v>
       </c>
       <c r="B29" t="n">
         <v>9</v>
       </c>
-      <c r="C29" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D29" s="6" t="n">
+      <c r="C29" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D29" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E29" t="n">
         <v>39</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="G29" s="9" t="n">
         <v>55.82</v>
       </c>
-      <c r="H29" s="5" t="n">
+      <c r="H29" s="9" t="n">
         <v>305.44</v>
       </c>
-      <c r="I29" s="5" t="n">
+      <c r="I29" s="9" t="n">
         <v>12636.69</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="8" t="n">
         <v>46502</v>
       </c>
       <c r="B30" t="n">
         <v>10</v>
       </c>
-      <c r="C30" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D30" s="6" t="n">
+      <c r="C30" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D30" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E30" t="n">
         <v>38</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G30" s="5" t="n">
+      <c r="G30" s="9" t="n">
         <v>54.5</v>
       </c>
-      <c r="H30" s="5" t="n">
+      <c r="H30" s="9" t="n">
         <v>306.75</v>
       </c>
-      <c r="I30" s="5" t="n">
+      <c r="I30" s="9" t="n">
         <v>12329.94</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="8" t="n">
         <v>46532</v>
       </c>
       <c r="B31" t="n">
         <v>11</v>
       </c>
-      <c r="C31" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D31" s="6" t="n">
+      <c r="C31" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D31" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E31" t="n">
         <v>37</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G31" s="5" t="n">
+      <c r="G31" s="9" t="n">
         <v>53.18</v>
       </c>
-      <c r="H31" s="5" t="n">
+      <c r="H31" s="9" t="n">
         <v>308.08</v>
       </c>
-      <c r="I31" s="5" t="n">
+      <c r="I31" s="9" t="n">
         <v>12021.86</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="8" t="n">
         <v>46563</v>
       </c>
       <c r="B32" t="n">
         <v>12</v>
       </c>
-      <c r="C32" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D32" s="6" t="n">
+      <c r="C32" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D32" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E32" t="n">
         <v>36</v>
       </c>
-      <c r="F32" s="5" t="n">
+      <c r="F32" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G32" s="5" t="n">
+      <c r="G32" s="9" t="n">
         <v>51.85</v>
       </c>
-      <c r="H32" s="5" t="n">
+      <c r="H32" s="9" t="n">
         <v>309.4</v>
       </c>
-      <c r="I32" s="5" t="n">
+      <c r="I32" s="9" t="n">
         <v>11712.46</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="8" t="n">
         <v>46593</v>
       </c>
       <c r="B33" t="n">
         <v>13</v>
       </c>
-      <c r="C33" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D33" s="6" t="n">
+      <c r="C33" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D33" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E33" t="n">
         <v>35</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F33" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="G33" s="9" t="n">
         <v>50.51</v>
       </c>
-      <c r="H33" s="5" t="n">
+      <c r="H33" s="9" t="n">
         <v>310.74</v>
       </c>
-      <c r="I33" s="5" t="n">
+      <c r="I33" s="9" t="n">
         <v>11401.72</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="A34" s="8" t="n">
         <v>46624</v>
       </c>
       <c r="B34" t="n">
         <v>14</v>
       </c>
-      <c r="C34" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D34" s="6" t="n">
+      <c r="C34" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D34" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E34" t="n">
         <v>34</v>
       </c>
-      <c r="F34" s="5" t="n">
+      <c r="F34" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G34" s="5" t="n">
+      <c r="G34" s="9" t="n">
         <v>49.17</v>
       </c>
-      <c r="H34" s="5" t="n">
+      <c r="H34" s="9" t="n">
         <v>312.08</v>
       </c>
-      <c r="I34" s="5" t="n">
+      <c r="I34" s="9" t="n">
         <v>11089.64</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n">
+      <c r="A35" s="8" t="n">
         <v>46655</v>
       </c>
       <c r="B35" t="n">
         <v>15</v>
       </c>
-      <c r="C35" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D35" s="6" t="n">
+      <c r="C35" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D35" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E35" t="n">
         <v>33</v>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="9" t="n">
         <v>47.83</v>
       </c>
-      <c r="H35" s="5" t="n">
+      <c r="H35" s="9" t="n">
         <v>313.43</v>
       </c>
-      <c r="I35" s="5" t="n">
+      <c r="I35" s="9" t="n">
         <v>10776.21</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="8" t="n">
         <v>46685</v>
       </c>
       <c r="B36" t="n">
         <v>16</v>
       </c>
-      <c r="C36" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D36" s="6" t="n">
+      <c r="C36" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D36" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E36" t="n">
         <v>32</v>
       </c>
-      <c r="F36" s="5" t="n">
+      <c r="F36" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G36" s="5" t="n">
+      <c r="G36" s="9" t="n">
         <v>46.48</v>
       </c>
-      <c r="H36" s="5" t="n">
+      <c r="H36" s="9" t="n">
         <v>314.78</v>
       </c>
-      <c r="I36" s="5" t="n">
+      <c r="I36" s="9" t="n">
         <v>10461.43</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n">
+      <c r="A37" s="8" t="n">
         <v>46716</v>
       </c>
       <c r="B37" t="n">
         <v>17</v>
       </c>
-      <c r="C37" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D37" s="6" t="n">
+      <c r="C37" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D37" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E37" t="n">
         <v>31</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F37" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="G37" s="9" t="n">
         <v>45.12</v>
       </c>
-      <c r="H37" s="5" t="n">
+      <c r="H37" s="9" t="n">
         <v>316.13</v>
       </c>
-      <c r="I37" s="5" t="n">
+      <c r="I37" s="9" t="n">
         <v>10145.3</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n">
+      <c r="A38" s="8" t="n">
         <v>46746</v>
       </c>
       <c r="B38" t="n">
         <v>18</v>
       </c>
-      <c r="C38" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D38" s="6" t="n">
+      <c r="C38" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D38" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E38" t="n">
         <v>30</v>
       </c>
-      <c r="F38" s="5" t="n">
+      <c r="F38" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G38" s="5" t="n">
+      <c r="G38" s="9" t="n">
         <v>43.76</v>
       </c>
-      <c r="H38" s="5" t="n">
+      <c r="H38" s="9" t="n">
         <v>317.5</v>
       </c>
-      <c r="I38" s="5" t="n">
+      <c r="I38" s="9" t="n">
         <v>9827.799999999999</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n">
+      <c r="A39" s="8" t="n">
         <v>46777</v>
       </c>
       <c r="B39" t="n">
         <v>19</v>
       </c>
-      <c r="C39" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D39" s="6" t="n">
+      <c r="C39" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D39" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E39" t="n">
         <v>29</v>
       </c>
-      <c r="F39" s="5" t="n">
+      <c r="F39" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G39" s="5" t="n">
+      <c r="G39" s="9" t="n">
         <v>42.39</v>
       </c>
-      <c r="H39" s="5" t="n">
+      <c r="H39" s="9" t="n">
         <v>318.87</v>
       </c>
-      <c r="I39" s="5" t="n">
+      <c r="I39" s="9" t="n">
         <v>9508.93</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n">
+      <c r="A40" s="8" t="n">
         <v>46808</v>
       </c>
       <c r="B40" t="n">
         <v>20</v>
       </c>
-      <c r="C40" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D40" s="6" t="n">
+      <c r="C40" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D40" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E40" t="n">
         <v>28</v>
       </c>
-      <c r="F40" s="5" t="n">
+      <c r="F40" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G40" s="5" t="n">
+      <c r="G40" s="9" t="n">
         <v>41.01</v>
       </c>
-      <c r="H40" s="5" t="n">
+      <c r="H40" s="9" t="n">
         <v>320.24</v>
       </c>
-      <c r="I40" s="5" t="n">
+      <c r="I40" s="9" t="n">
         <v>9188.690000000001</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n">
+      <c r="A41" s="8" t="n">
         <v>46837</v>
       </c>
       <c r="B41" t="n">
         <v>21</v>
       </c>
-      <c r="C41" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D41" s="6" t="n">
+      <c r="C41" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D41" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E41" t="n">
         <v>27</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F41" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G41" s="5" t="n">
+      <c r="G41" s="9" t="n">
         <v>39.63</v>
       </c>
-      <c r="H41" s="5" t="n">
+      <c r="H41" s="9" t="n">
         <v>321.62</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I41" s="9" t="n">
         <v>8867.07</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n">
+      <c r="A42" s="8" t="n">
         <v>46868</v>
       </c>
       <c r="B42" t="n">
         <v>22</v>
       </c>
-      <c r="C42" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D42" s="6" t="n">
+      <c r="C42" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D42" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E42" t="n">
         <v>26</v>
       </c>
-      <c r="F42" s="5" t="n">
+      <c r="F42" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G42" s="5" t="n">
+      <c r="G42" s="9" t="n">
         <v>38.24</v>
       </c>
-      <c r="H42" s="5" t="n">
+      <c r="H42" s="9" t="n">
         <v>323.01</v>
       </c>
-      <c r="I42" s="5" t="n">
+      <c r="I42" s="9" t="n">
         <v>8544.059999999999</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n">
+      <c r="A43" s="8" t="n">
         <v>46898</v>
       </c>
       <c r="B43" t="n">
         <v>23</v>
       </c>
-      <c r="C43" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D43" s="6" t="n">
+      <c r="C43" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D43" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E43" t="n">
         <v>25</v>
       </c>
-      <c r="F43" s="5" t="n">
+      <c r="F43" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G43" s="5" t="n">
+      <c r="G43" s="9" t="n">
         <v>36.85</v>
       </c>
-      <c r="H43" s="5" t="n">
+      <c r="H43" s="9" t="n">
         <v>324.4</v>
       </c>
-      <c r="I43" s="5" t="n">
+      <c r="I43" s="9" t="n">
         <v>8219.65</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="n">
+      <c r="A44" s="8" t="n">
         <v>46929</v>
       </c>
       <c r="B44" t="n">
         <v>24</v>
       </c>
-      <c r="C44" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D44" s="6" t="n">
+      <c r="C44" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D44" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E44" t="n">
         <v>24</v>
       </c>
-      <c r="F44" s="5" t="n">
+      <c r="F44" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G44" s="5" t="n">
+      <c r="G44" s="9" t="n">
         <v>35.45</v>
       </c>
-      <c r="H44" s="5" t="n">
+      <c r="H44" s="9" t="n">
         <v>325.8</v>
       </c>
-      <c r="I44" s="5" t="n">
+      <c r="I44" s="9" t="n">
         <v>7893.85</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n">
+      <c r="A45" s="8" t="n">
         <v>46959</v>
       </c>
       <c r="B45" t="n">
         <v>25</v>
       </c>
-      <c r="C45" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D45" s="6" t="n">
+      <c r="C45" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D45" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E45" t="n">
         <v>23</v>
       </c>
-      <c r="F45" s="5" t="n">
+      <c r="F45" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G45" s="5" t="n">
+      <c r="G45" s="9" t="n">
         <v>34.05</v>
       </c>
-      <c r="H45" s="5" t="n">
+      <c r="H45" s="9" t="n">
         <v>327.21</v>
       </c>
-      <c r="I45" s="5" t="n">
+      <c r="I45" s="9" t="n">
         <v>7566.64</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="A46" s="8" t="n">
         <v>46990</v>
       </c>
       <c r="B46" t="n">
         <v>26</v>
       </c>
-      <c r="C46" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D46" s="6" t="n">
+      <c r="C46" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D46" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E46" t="n">
         <v>22</v>
       </c>
-      <c r="F46" s="5" t="n">
+      <c r="F46" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G46" s="5" t="n">
+      <c r="G46" s="9" t="n">
         <v>32.63</v>
       </c>
-      <c r="H46" s="5" t="n">
+      <c r="H46" s="9" t="n">
         <v>328.62</v>
       </c>
-      <c r="I46" s="5" t="n">
+      <c r="I46" s="9" t="n">
         <v>7238.02</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="n">
+      <c r="A47" s="8" t="n">
         <v>47021</v>
       </c>
       <c r="B47" t="n">
         <v>27</v>
       </c>
-      <c r="C47" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D47" s="6" t="n">
+      <c r="C47" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D47" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E47" t="n">
         <v>21</v>
       </c>
-      <c r="F47" s="5" t="n">
+      <c r="F47" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G47" s="5" t="n">
+      <c r="G47" s="9" t="n">
         <v>31.22</v>
       </c>
-      <c r="H47" s="5" t="n">
+      <c r="H47" s="9" t="n">
         <v>330.04</v>
       </c>
-      <c r="I47" s="5" t="n">
+      <c r="I47" s="9" t="n">
         <v>6907.98</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n">
+      <c r="A48" s="8" t="n">
         <v>47051</v>
       </c>
       <c r="B48" t="n">
         <v>28</v>
       </c>
-      <c r="C48" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D48" s="6" t="n">
+      <c r="C48" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D48" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E48" t="n">
         <v>20</v>
       </c>
-      <c r="F48" s="5" t="n">
+      <c r="F48" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G48" s="5" t="n">
+      <c r="G48" s="9" t="n">
         <v>29.79</v>
       </c>
-      <c r="H48" s="5" t="n">
+      <c r="H48" s="9" t="n">
         <v>331.46</v>
       </c>
-      <c r="I48" s="5" t="n">
+      <c r="I48" s="9" t="n">
         <v>6576.52</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="n">
+      <c r="A49" s="8" t="n">
         <v>47082</v>
       </c>
       <c r="B49" t="n">
         <v>29</v>
       </c>
-      <c r="C49" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D49" s="6" t="n">
+      <c r="C49" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D49" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E49" t="n">
         <v>19</v>
       </c>
-      <c r="F49" s="5" t="n">
+      <c r="F49" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G49" s="5" t="n">
+      <c r="G49" s="9" t="n">
         <v>28.36</v>
       </c>
-      <c r="H49" s="5" t="n">
+      <c r="H49" s="9" t="n">
         <v>332.89</v>
       </c>
-      <c r="I49" s="5" t="n">
+      <c r="I49" s="9" t="n">
         <v>6243.63</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n">
+      <c r="A50" s="8" t="n">
         <v>47112</v>
       </c>
       <c r="B50" t="n">
         <v>30</v>
       </c>
-      <c r="C50" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D50" s="6" t="n">
+      <c r="C50" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D50" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E50" t="n">
         <v>18</v>
       </c>
-      <c r="F50" s="5" t="n">
+      <c r="F50" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G50" s="5" t="n">
+      <c r="G50" s="9" t="n">
         <v>26.93</v>
       </c>
-      <c r="H50" s="5" t="n">
+      <c r="H50" s="9" t="n">
         <v>334.33</v>
       </c>
-      <c r="I50" s="5" t="n">
+      <c r="I50" s="9" t="n">
         <v>5909.31</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n">
+      <c r="A51" s="8" t="n">
         <v>47143</v>
       </c>
       <c r="B51" t="n">
         <v>31</v>
       </c>
-      <c r="C51" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D51" s="6" t="n">
+      <c r="C51" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D51" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E51" t="n">
         <v>17</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F51" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G51" s="5" t="n">
+      <c r="G51" s="9" t="n">
         <v>25.49</v>
       </c>
-      <c r="H51" s="5" t="n">
+      <c r="H51" s="9" t="n">
         <v>335.77</v>
       </c>
-      <c r="I51" s="5" t="n">
+      <c r="I51" s="9" t="n">
         <v>5573.54</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="n">
+      <c r="A52" s="8" t="n">
         <v>47174</v>
       </c>
       <c r="B52" t="n">
         <v>32</v>
       </c>
-      <c r="C52" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D52" s="6" t="n">
+      <c r="C52" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D52" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E52" t="n">
         <v>16</v>
       </c>
-      <c r="F52" s="5" t="n">
+      <c r="F52" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G52" s="5" t="n">
+      <c r="G52" s="9" t="n">
         <v>24.04</v>
       </c>
-      <c r="H52" s="5" t="n">
+      <c r="H52" s="9" t="n">
         <v>337.22</v>
       </c>
-      <c r="I52" s="5" t="n">
+      <c r="I52" s="9" t="n">
         <v>5236.32</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="n">
+      <c r="A53" s="8" t="n">
         <v>47202</v>
       </c>
       <c r="B53" t="n">
         <v>33</v>
       </c>
-      <c r="C53" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D53" s="6" t="n">
+      <c r="C53" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D53" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E53" t="n">
         <v>15</v>
       </c>
-      <c r="F53" s="5" t="n">
+      <c r="F53" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G53" s="5" t="n">
+      <c r="G53" s="9" t="n">
         <v>22.58</v>
       </c>
-      <c r="H53" s="5" t="n">
+      <c r="H53" s="9" t="n">
         <v>338.67</v>
       </c>
-      <c r="I53" s="5" t="n">
+      <c r="I53" s="9" t="n">
         <v>4897.65</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="n">
+      <c r="A54" s="8" t="n">
         <v>47233</v>
       </c>
       <c r="B54" t="n">
         <v>34</v>
       </c>
-      <c r="C54" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D54" s="6" t="n">
+      <c r="C54" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D54" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E54" t="n">
         <v>14</v>
       </c>
-      <c r="F54" s="5" t="n">
+      <c r="F54" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G54" s="5" t="n">
+      <c r="G54" s="9" t="n">
         <v>21.12</v>
       </c>
-      <c r="H54" s="5" t="n">
+      <c r="H54" s="9" t="n">
         <v>340.13</v>
       </c>
-      <c r="I54" s="5" t="n">
+      <c r="I54" s="9" t="n">
         <v>4557.52</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="n">
+      <c r="A55" s="8" t="n">
         <v>47263</v>
       </c>
       <c r="B55" t="n">
         <v>35</v>
       </c>
-      <c r="C55" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D55" s="6" t="n">
+      <c r="C55" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D55" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E55" t="n">
         <v>13</v>
       </c>
-      <c r="F55" s="5" t="n">
+      <c r="F55" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G55" s="5" t="n">
+      <c r="G55" s="9" t="n">
         <v>19.66</v>
       </c>
-      <c r="H55" s="5" t="n">
+      <c r="H55" s="9" t="n">
         <v>341.6</v>
       </c>
-      <c r="I55" s="5" t="n">
+      <c r="I55" s="9" t="n">
         <v>4215.92</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="n">
+      <c r="A56" s="8" t="n">
         <v>47294</v>
       </c>
       <c r="B56" t="n">
         <v>36</v>
       </c>
-      <c r="C56" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D56" s="6" t="n">
+      <c r="C56" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D56" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E56" t="n">
         <v>12</v>
       </c>
-      <c r="F56" s="5" t="n">
+      <c r="F56" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G56" s="5" t="n">
+      <c r="G56" s="9" t="n">
         <v>18.18</v>
       </c>
-      <c r="H56" s="5" t="n">
+      <c r="H56" s="9" t="n">
         <v>343.07</v>
       </c>
-      <c r="I56" s="5" t="n">
+      <c r="I56" s="9" t="n">
         <v>3872.85</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="n">
+      <c r="A57" s="8" t="n">
         <v>47324</v>
       </c>
       <c r="B57" t="n">
         <v>37</v>
       </c>
-      <c r="C57" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D57" s="6" t="n">
+      <c r="C57" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D57" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E57" t="n">
         <v>11</v>
       </c>
-      <c r="F57" s="5" t="n">
+      <c r="F57" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G57" s="5" t="n">
+      <c r="G57" s="9" t="n">
         <v>16.7</v>
       </c>
-      <c r="H57" s="5" t="n">
+      <c r="H57" s="9" t="n">
         <v>344.55</v>
       </c>
-      <c r="I57" s="5" t="n">
+      <c r="I57" s="9" t="n">
         <v>3528.3</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="n">
+      <c r="A58" s="8" t="n">
         <v>47355</v>
       </c>
       <c r="B58" t="n">
         <v>38</v>
       </c>
-      <c r="C58" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D58" s="6" t="n">
+      <c r="C58" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D58" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E58" t="n">
         <v>10</v>
       </c>
-      <c r="F58" s="5" t="n">
+      <c r="F58" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G58" s="5" t="n">
+      <c r="G58" s="9" t="n">
         <v>15.22</v>
       </c>
-      <c r="H58" s="5" t="n">
+      <c r="H58" s="9" t="n">
         <v>346.04</v>
       </c>
-      <c r="I58" s="5" t="n">
+      <c r="I58" s="9" t="n">
         <v>3182.27</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="n">
+      <c r="A59" s="8" t="n">
         <v>47386</v>
       </c>
       <c r="B59" t="n">
         <v>39</v>
       </c>
-      <c r="C59" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D59" s="6" t="n">
+      <c r="C59" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D59" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E59" t="n">
         <v>9</v>
       </c>
-      <c r="F59" s="5" t="n">
+      <c r="F59" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G59" s="5" t="n">
+      <c r="G59" s="9" t="n">
         <v>13.72</v>
       </c>
-      <c r="H59" s="5" t="n">
+      <c r="H59" s="9" t="n">
         <v>347.53</v>
       </c>
-      <c r="I59" s="5" t="n">
+      <c r="I59" s="9" t="n">
         <v>2834.74</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="n">
+      <c r="A60" s="8" t="n">
         <v>47416</v>
       </c>
       <c r="B60" t="n">
         <v>40</v>
       </c>
-      <c r="C60" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D60" s="6" t="n">
+      <c r="C60" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D60" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E60" t="n">
         <v>8</v>
       </c>
-      <c r="F60" s="5" t="n">
+      <c r="F60" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G60" s="5" t="n">
+      <c r="G60" s="9" t="n">
         <v>12.23</v>
       </c>
-      <c r="H60" s="5" t="n">
+      <c r="H60" s="9" t="n">
         <v>349.03</v>
       </c>
-      <c r="I60" s="5" t="n">
+      <c r="I60" s="9" t="n">
         <v>2485.71</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="n">
+      <c r="A61" s="8" t="n">
         <v>47447</v>
       </c>
       <c r="B61" t="n">
         <v>41</v>
       </c>
-      <c r="C61" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D61" s="6" t="n">
+      <c r="C61" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D61" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E61" t="n">
         <v>7</v>
       </c>
-      <c r="F61" s="5" t="n">
+      <c r="F61" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G61" s="5" t="n">
+      <c r="G61" s="9" t="n">
         <v>10.72</v>
       </c>
-      <c r="H61" s="5" t="n">
+      <c r="H61" s="9" t="n">
         <v>350.53</v>
       </c>
-      <c r="I61" s="5" t="n">
+      <c r="I61" s="9" t="n">
         <v>2135.18</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="n">
+      <c r="A62" s="8" t="n">
         <v>47477</v>
       </c>
       <c r="B62" t="n">
         <v>42</v>
       </c>
-      <c r="C62" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D62" s="6" t="n">
+      <c r="C62" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D62" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E62" t="n">
         <v>6</v>
       </c>
-      <c r="F62" s="5" t="n">
+      <c r="F62" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G62" s="5" t="n">
+      <c r="G62" s="9" t="n">
         <v>9.210000000000001</v>
       </c>
-      <c r="H62" s="5" t="n">
+      <c r="H62" s="9" t="n">
         <v>352.04</v>
       </c>
-      <c r="I62" s="5" t="n">
+      <c r="I62" s="9" t="n">
         <v>1783.13</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="n">
+      <c r="A63" s="8" t="n">
         <v>47508</v>
       </c>
       <c r="B63" t="n">
         <v>43</v>
       </c>
-      <c r="C63" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D63" s="6" t="n">
+      <c r="C63" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D63" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E63" t="n">
         <v>5</v>
       </c>
-      <c r="F63" s="5" t="n">
+      <c r="F63" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G63" s="5" t="n">
+      <c r="G63" s="9" t="n">
         <v>7.69</v>
       </c>
-      <c r="H63" s="5" t="n">
+      <c r="H63" s="9" t="n">
         <v>353.56</v>
       </c>
-      <c r="I63" s="5" t="n">
+      <c r="I63" s="9" t="n">
         <v>1429.57</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="n">
+      <c r="A64" s="8" t="n">
         <v>47539</v>
       </c>
       <c r="B64" t="n">
         <v>44</v>
       </c>
-      <c r="C64" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D64" s="6" t="n">
+      <c r="C64" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D64" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E64" t="n">
         <v>4</v>
       </c>
-      <c r="F64" s="5" t="n">
+      <c r="F64" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G64" s="5" t="n">
+      <c r="G64" s="9" t="n">
         <v>6.17</v>
       </c>
-      <c r="H64" s="5" t="n">
+      <c r="H64" s="9" t="n">
         <v>355.09</v>
       </c>
-      <c r="I64" s="5" t="n">
+      <c r="I64" s="9" t="n">
         <v>1074.48</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="n">
+      <c r="A65" s="8" t="n">
         <v>47567</v>
       </c>
       <c r="B65" t="n">
         <v>45</v>
       </c>
-      <c r="C65" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D65" s="6" t="n">
+      <c r="C65" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D65" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E65" t="n">
         <v>3</v>
       </c>
-      <c r="F65" s="5" t="n">
+      <c r="F65" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G65" s="5" t="n">
+      <c r="G65" s="9" t="n">
         <v>4.63</v>
       </c>
-      <c r="H65" s="5" t="n">
+      <c r="H65" s="9" t="n">
         <v>356.62</v>
       </c>
-      <c r="I65" s="5" t="n">
+      <c r="I65" s="9" t="n">
         <v>717.86</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="n">
+      <c r="A66" s="8" t="n">
         <v>47598</v>
       </c>
       <c r="B66" t="n">
         <v>46</v>
       </c>
-      <c r="C66" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D66" s="6" t="n">
+      <c r="C66" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D66" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E66" t="n">
         <v>2</v>
       </c>
-      <c r="F66" s="5" t="n">
+      <c r="F66" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G66" s="5" t="n">
+      <c r="G66" s="9" t="n">
         <v>3.1</v>
       </c>
-      <c r="H66" s="5" t="n">
+      <c r="H66" s="9" t="n">
         <v>358.16</v>
       </c>
-      <c r="I66" s="5" t="n">
+      <c r="I66" s="9" t="n">
         <v>359.7</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="n">
+      <c r="A67" s="8" t="n">
         <v>47628</v>
       </c>
       <c r="B67" t="n">
         <v>47</v>
       </c>
-      <c r="C67" s="6" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D67" s="6" t="n">
+      <c r="C67" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D67" s="10" t="n">
         <v>0.00431288</v>
       </c>
       <c r="E67" t="n">
         <v>1</v>
       </c>
-      <c r="F67" s="5" t="n">
+      <c r="F67" s="9" t="n">
         <v>361.25</v>
       </c>
-      <c r="G67" s="5" t="n">
+      <c r="G67" s="9" t="n">
         <v>1.55</v>
       </c>
-      <c r="H67" s="5" t="n">
+      <c r="H67" s="9" t="n">
         <v>359.7</v>
       </c>
-      <c r="I67" s="5" t="n">
+      <c r="I67" s="9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>